<commit_message>
added a clear whole pipeline demonstration notebook(08)
</commit_message>
<xml_diff>
--- a/results/tables/03_env_driven_taxa_clusters/table1_rda_axes_summary.xlsx
+++ b/results/tables/03_env_driven_taxa_clusters/table1_rda_axes_summary.xlsx
@@ -475,23 +475,23 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.0212431472997022</v>
+        <v>0.03435113210021093</v>
       </c>
       <c r="D2" t="n">
-        <v>38.94440718155573</v>
+        <v>52.93113550334336</v>
       </c>
       <c r="E2" t="n">
-        <v>38.94440718155573</v>
+        <v>52.93113550334336</v>
       </c>
       <c r="F2" t="n">
-        <v>2.93947000206741</v>
+        <v>6.274855610434186</v>
       </c>
       <c r="G2" t="n">
-        <v>0.135</v>
+        <v>0.001</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>ns</t>
+          <t>**</t>
         </is>
       </c>
     </row>
@@ -505,19 +505,19 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.01482919321081708</v>
+        <v>0.01208337310482697</v>
       </c>
       <c r="D3" t="n">
-        <v>27.18590284331918</v>
+        <v>18.61908531233309</v>
       </c>
       <c r="E3" t="n">
-        <v>66.13031002487492</v>
+        <v>71.55022081567645</v>
       </c>
       <c r="F3" t="n">
-        <v>2.051954354177527</v>
+        <v>2.207246657798724</v>
       </c>
       <c r="G3" t="n">
-        <v>0.645</v>
+        <v>0.551</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -535,19 +535,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.007163093911575461</v>
+        <v>0.007207702058702983</v>
       </c>
       <c r="D4" t="n">
-        <v>13.13187928495079</v>
+        <v>11.10623816484324</v>
       </c>
       <c r="E4" t="n">
-        <v>79.2621893098257</v>
+        <v>82.6564589805197</v>
       </c>
       <c r="F4" t="n">
-        <v>0.9911760897766286</v>
+        <v>1.31661715164004</v>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>0.986</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -565,19 +565,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.005253273026993101</v>
+        <v>0.005759433985013814</v>
       </c>
       <c r="D5" t="n">
-        <v>9.630663522347801</v>
+        <v>8.87462398019351</v>
       </c>
       <c r="E5" t="n">
-        <v>88.8928528321735</v>
+        <v>91.53108296071321</v>
       </c>
       <c r="F5" t="n">
-        <v>0.7269091654668588</v>
+        <v>1.05206479216932</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>0.998</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -595,16 +595,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.004344218967067539</v>
+        <v>0.003353185157688655</v>
       </c>
       <c r="D6" t="n">
-        <v>7.964122733437312</v>
+        <v>5.166871864124912</v>
       </c>
       <c r="E6" t="n">
-        <v>96.85697556561081</v>
+        <v>96.69795482483812</v>
       </c>
       <c r="F6" t="n">
-        <v>0.6011209711983835</v>
+        <v>0.6125199203963964</v>
       </c>
       <c r="G6" t="n">
         <v>1</v>
@@ -625,16 +625,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.001714436959202559</v>
+        <v>0.00214295402760981</v>
       </c>
       <c r="D7" t="n">
-        <v>3.143024434389189</v>
+        <v>3.302045175161891</v>
       </c>
       <c r="E7" t="n">
         <v>100</v>
       </c>
       <c r="F7" t="n">
-        <v>0.2372311381601275</v>
+        <v>0.3914493142124822</v>
       </c>
       <c r="G7" t="n">
         <v>1</v>

</xml_diff>